<commit_message>
Updated Data with CTA Stop Update Report
</commit_message>
<xml_diff>
--- a/Data/Data Second Assignment/DataPhase2Horowitz.xlsx
+++ b/Data/Data Second Assignment/DataPhase2Horowitz.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/14270eef50ba1d21/Documents/GitHub/CS424_Fall2016_Project/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/14270eef50ba1d21/Documents/GitHub/CS424_Fall2016_Project/Data/Data Second Assignment/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="169" documentId="8_{43A70E10-A03E-4ECA-80A8-269F31A6B0A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B063C2D-8829-4639-9B21-2568A0BEDC00}"/>
+  <xr:revisionPtr revIDLastSave="183" documentId="8_{43A70E10-A03E-4ECA-80A8-269F31A6B0A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A38AE64F-6297-456C-8A27-90F046BF83AB}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{AC6E6D69-EF37-40C5-A55F-0E10EFBF8A2F}"/>
+    <workbookView xWindow="1152" yWindow="1152" windowWidth="17280" windowHeight="8880" xr2:uid="{AC6E6D69-EF37-40C5-A55F-0E10EFBF8A2F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="39">
   <si>
     <t>Observation ID</t>
   </si>
@@ -153,6 +153,9 @@
   </si>
   <si>
     <t>N</t>
+  </si>
+  <si>
+    <t>Stop ID</t>
   </si>
 </sst>
 </file>
@@ -160,7 +163,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="h:mm;@"/>
+    <numFmt numFmtId="164" formatCode="h:mm;@"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -199,13 +202,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -221,6 +223,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -540,24 +546,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42D2C34E-AD17-4563-BB06-176FFE88B011}">
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:M34"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.21875" customWidth="1"/>
     <col min="3" max="3" width="23.44140625" customWidth="1"/>
     <col min="4" max="4" width="23.88671875" customWidth="1"/>
-    <col min="5" max="5" width="26.6640625" customWidth="1"/>
-    <col min="6" max="6" width="19.5546875" customWidth="1"/>
-    <col min="7" max="7" width="25.88671875" customWidth="1"/>
-    <col min="8" max="8" width="23.77734375" customWidth="1"/>
-    <col min="9" max="9" width="25.44140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="26.33203125" customWidth="1"/>
-    <col min="11" max="11" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="65.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="26.6640625" customWidth="1"/>
+    <col min="7" max="7" width="19.5546875" customWidth="1"/>
+    <col min="8" max="8" width="25.88671875" customWidth="1"/>
+    <col min="9" max="9" width="23.77734375" customWidth="1"/>
+    <col min="10" max="10" width="25.44140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="26.33203125" customWidth="1"/>
+    <col min="12" max="12" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="65.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -574,28 +580,31 @@
         <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -611,29 +620,32 @@
       <c r="E2" t="s">
         <v>13</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2">
+        <v>5792</v>
+      </c>
+      <c r="G2" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="1">
+      <c r="H2" s="1">
         <v>0.40694444444444444</v>
       </c>
-      <c r="H2" s="1">
+      <c r="I2" s="1">
         <v>0.40347222222222223</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>15</v>
       </c>
-      <c r="J2">
+      <c r="K2">
         <v>15</v>
       </c>
-      <c r="K2">
+      <c r="L2">
         <v>2</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -649,29 +661,32 @@
       <c r="E3" t="s">
         <v>13</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3">
+        <v>5792</v>
+      </c>
+      <c r="G3" t="s">
         <v>14</v>
       </c>
-      <c r="G3" s="1">
+      <c r="H3" s="1">
         <v>0.41666666666666669</v>
       </c>
-      <c r="H3" s="1">
+      <c r="I3" s="1">
         <v>0.40486111111111112</v>
       </c>
-      <c r="I3">
+      <c r="J3">
         <v>2</v>
       </c>
-      <c r="J3">
+      <c r="K3">
         <v>14</v>
       </c>
-      <c r="K3">
+      <c r="L3">
         <v>13</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -687,29 +702,32 @@
       <c r="E4" t="s">
         <v>13</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4">
+        <v>5792</v>
+      </c>
+      <c r="G4" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="1">
+      <c r="H4" s="1">
         <v>0.41319444444444442</v>
       </c>
-      <c r="H4" s="1">
+      <c r="I4" s="1">
         <v>0.41388888888888886</v>
       </c>
-      <c r="I4">
+      <c r="J4">
         <v>13</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <v>11</v>
       </c>
-      <c r="K4">
+      <c r="L4">
         <v>10</v>
       </c>
-      <c r="L4" t="s">
+      <c r="M4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -725,29 +743,32 @@
       <c r="E5" t="s">
         <v>13</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5">
+        <v>5792</v>
+      </c>
+      <c r="G5" t="s">
         <v>14</v>
       </c>
-      <c r="G5" s="1">
+      <c r="H5" s="1">
         <v>0.42083333333333334</v>
       </c>
-      <c r="H5" s="1">
+      <c r="I5" s="1">
         <v>0.4201388888888889</v>
       </c>
-      <c r="I5">
+      <c r="J5">
         <v>10</v>
       </c>
-      <c r="J5">
+      <c r="K5">
         <v>12</v>
       </c>
-      <c r="K5">
+      <c r="L5">
         <v>8</v>
       </c>
-      <c r="L5" t="s">
+      <c r="M5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -763,29 +784,32 @@
       <c r="E6" t="s">
         <v>13</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6">
+        <v>5792</v>
+      </c>
+      <c r="G6" t="s">
         <v>14</v>
       </c>
-      <c r="G6" s="1">
+      <c r="H6" s="1">
         <v>0.42708333333333331</v>
       </c>
-      <c r="H6" s="1">
+      <c r="I6" s="1">
         <v>0.42638888888888887</v>
       </c>
-      <c r="I6">
+      <c r="J6">
         <v>8</v>
       </c>
-      <c r="J6">
+      <c r="K6">
         <v>13</v>
       </c>
-      <c r="K6" t="s">
+      <c r="L6" t="s">
         <v>15</v>
       </c>
-      <c r="L6" t="s">
+      <c r="M6" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -801,29 +825,32 @@
       <c r="E7" t="s">
         <v>21</v>
       </c>
-      <c r="F7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G7" s="1">
-        <v>0.73888888888888893</v>
+      <c r="F7">
+        <v>771</v>
+      </c>
+      <c r="G7" t="s">
+        <v>22</v>
       </c>
       <c r="H7" s="1">
         <v>0.73888888888888893</v>
       </c>
-      <c r="I7">
+      <c r="I7" s="1">
+        <v>0.73888888888888893</v>
+      </c>
+      <c r="J7">
         <v>21</v>
       </c>
-      <c r="J7">
-        <v>0</v>
-      </c>
       <c r="K7">
         <v>0</v>
       </c>
-      <c r="L7" t="s">
+      <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="M7" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -839,29 +866,32 @@
       <c r="E8" t="s">
         <v>21</v>
       </c>
-      <c r="F8" t="s">
-        <v>22</v>
-      </c>
-      <c r="G8" s="1">
+      <c r="F8">
+        <v>771</v>
+      </c>
+      <c r="G8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H8" s="1">
         <v>0.73888888888888893</v>
       </c>
-      <c r="H8" s="1">
+      <c r="I8" s="1">
         <v>0.73958333333333337</v>
       </c>
-      <c r="I8">
-        <v>0</v>
-      </c>
       <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
         <v>4</v>
       </c>
-      <c r="K8">
+      <c r="L8">
         <v>1</v>
       </c>
-      <c r="L8" t="s">
+      <c r="M8" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -877,29 +907,32 @@
       <c r="E9" t="s">
         <v>21</v>
       </c>
-      <c r="F9" t="s">
-        <v>22</v>
-      </c>
-      <c r="G9" s="1">
+      <c r="F9">
+        <v>771</v>
+      </c>
+      <c r="G9" t="s">
+        <v>22</v>
+      </c>
+      <c r="H9" s="1">
         <v>0.74861111111111112</v>
       </c>
-      <c r="H9" s="1">
+      <c r="I9" s="1">
         <v>0.74027777777777781</v>
       </c>
-      <c r="I9">
+      <c r="J9">
         <v>1</v>
       </c>
-      <c r="J9">
+      <c r="K9">
         <v>10</v>
       </c>
-      <c r="K9" t="s">
+      <c r="L9" t="s">
         <v>15</v>
       </c>
-      <c r="L9" t="s">
+      <c r="M9" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -915,29 +948,32 @@
       <c r="E10" t="s">
         <v>27</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10" t="s">
         <v>29</v>
       </c>
-      <c r="G10" s="4">
+      <c r="H10" s="4">
         <v>0.62638888888888888</v>
       </c>
-      <c r="H10" s="1">
+      <c r="I10" s="1">
         <v>0.62430555555555556</v>
       </c>
-      <c r="I10" t="s">
+      <c r="J10" t="s">
         <v>15</v>
       </c>
-      <c r="J10">
+      <c r="K10">
         <v>4</v>
       </c>
-      <c r="K10">
+      <c r="L10">
         <v>5</v>
       </c>
-      <c r="L10" t="s">
+      <c r="M10" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -953,29 +989,32 @@
       <c r="E11" t="s">
         <v>27</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="G11" t="s">
         <v>29</v>
-      </c>
-      <c r="G11" s="1">
-        <v>0.62708333333333333</v>
       </c>
       <c r="H11" s="1">
         <v>0.62708333333333333</v>
       </c>
-      <c r="I11" t="s">
+      <c r="I11" s="1">
+        <v>0.62708333333333333</v>
+      </c>
+      <c r="J11" t="s">
         <v>15</v>
-      </c>
-      <c r="J11">
-        <v>3</v>
       </c>
       <c r="K11">
         <v>3</v>
       </c>
-      <c r="L11" t="s">
+      <c r="L11">
+        <v>3</v>
+      </c>
+      <c r="M11" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -991,26 +1030,29 @@
       <c r="E12" t="s">
         <v>27</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12" t="s">
         <v>29</v>
       </c>
-      <c r="G12" s="1">
+      <c r="H12" s="1">
         <v>0.62847222222222221</v>
       </c>
-      <c r="H12" s="1">
+      <c r="I12" s="1">
         <v>0.62777777777777777</v>
       </c>
-      <c r="I12">
+      <c r="J12">
         <v>5</v>
       </c>
-      <c r="J12">
+      <c r="K12">
         <v>7</v>
       </c>
-      <c r="K12">
+      <c r="L12">
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1026,26 +1068,29 @@
       <c r="E13" t="s">
         <v>27</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13" t="s">
         <v>29</v>
       </c>
-      <c r="G13" s="1">
+      <c r="H13" s="1">
         <v>0.6333333333333333</v>
       </c>
-      <c r="H13" s="1">
+      <c r="I13" s="1">
         <v>0.62916666666666665</v>
       </c>
-      <c r="I13">
+      <c r="J13">
         <v>2</v>
       </c>
-      <c r="J13">
+      <c r="K13">
         <v>7</v>
       </c>
-      <c r="K13">
+      <c r="L13">
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1061,26 +1106,29 @@
       <c r="E14" t="s">
         <v>27</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="G14" t="s">
         <v>29</v>
       </c>
-      <c r="G14" s="1">
+      <c r="H14" s="1">
         <v>0.6333333333333333</v>
       </c>
-      <c r="H14" s="1">
+      <c r="I14" s="1">
         <v>0.63541666666666663</v>
       </c>
-      <c r="I14">
+      <c r="J14">
         <v>7</v>
       </c>
-      <c r="J14">
+      <c r="K14">
         <v>10</v>
       </c>
-      <c r="K14">
+      <c r="L14">
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1096,29 +1144,32 @@
       <c r="E15" t="s">
         <v>27</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15">
+        <v>0</v>
+      </c>
+      <c r="G15" t="s">
         <v>29</v>
       </c>
-      <c r="G15" s="1">
+      <c r="H15" s="1">
         <v>0.64027777777777772</v>
       </c>
-      <c r="H15" s="1">
+      <c r="I15" s="1">
         <v>0.63680555555555551</v>
       </c>
-      <c r="I15">
+      <c r="J15">
         <v>1</v>
       </c>
-      <c r="J15">
+      <c r="K15">
         <v>10</v>
       </c>
-      <c r="K15">
+      <c r="L15">
         <v>1</v>
       </c>
-      <c r="L15" t="s">
+      <c r="M15" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1134,29 +1185,32 @@
       <c r="E16" t="s">
         <v>27</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16">
+        <v>0</v>
+      </c>
+      <c r="G16" t="s">
         <v>29</v>
       </c>
-      <c r="G16" s="1">
+      <c r="H16" s="1">
         <v>0.64722222222222225</v>
       </c>
-      <c r="H16" s="1">
+      <c r="I16" s="1">
         <v>0.63749999999999996</v>
       </c>
-      <c r="I16">
+      <c r="J16">
         <v>1</v>
       </c>
-      <c r="J16">
+      <c r="K16">
         <v>5</v>
       </c>
-      <c r="K16">
+      <c r="L16">
         <v>6</v>
       </c>
-      <c r="L16" t="s">
+      <c r="M16" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1172,26 +1226,29 @@
       <c r="E17" t="s">
         <v>27</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17">
+        <v>0</v>
+      </c>
+      <c r="G17" t="s">
         <v>29</v>
       </c>
-      <c r="G17" s="1">
+      <c r="H17" s="1">
         <v>0.6381944444444444</v>
       </c>
-      <c r="H17" s="1">
+      <c r="I17" s="1">
         <v>0.64027777777777772</v>
       </c>
-      <c r="I17">
+      <c r="J17">
         <v>16</v>
       </c>
-      <c r="J17">
+      <c r="K17">
         <v>5</v>
       </c>
-      <c r="K17">
+      <c r="L17">
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1207,26 +1264,29 @@
       <c r="E18" t="s">
         <v>27</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F18">
+        <v>0</v>
+      </c>
+      <c r="G18" t="s">
         <v>29</v>
       </c>
-      <c r="G18" s="1">
+      <c r="H18" s="1">
         <v>0.64375000000000004</v>
       </c>
-      <c r="H18" s="1">
+      <c r="I18" s="1">
         <v>0.64444444444444449</v>
-      </c>
-      <c r="I18">
-        <v>10</v>
       </c>
       <c r="J18">
         <v>10</v>
       </c>
-      <c r="K18" t="s">
+      <c r="K18">
+        <v>10</v>
+      </c>
+      <c r="L18" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1242,29 +1302,32 @@
       <c r="E19" t="s">
         <v>27</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F19">
+        <v>0</v>
+      </c>
+      <c r="G19" t="s">
         <v>29</v>
       </c>
-      <c r="G19" s="1">
+      <c r="H19" s="1">
         <v>0.64027777777777772</v>
       </c>
-      <c r="H19" s="1">
+      <c r="I19" s="1">
         <v>0.64513888888888893</v>
       </c>
-      <c r="I19">
+      <c r="J19">
         <v>7</v>
       </c>
-      <c r="J19">
+      <c r="K19">
         <v>4</v>
       </c>
-      <c r="K19">
-        <v>0</v>
-      </c>
-      <c r="L19" t="s">
+      <c r="L19">
+        <v>0</v>
+      </c>
+      <c r="M19" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1280,29 +1343,32 @@
       <c r="E20" t="s">
         <v>27</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F20">
+        <v>0</v>
+      </c>
+      <c r="G20" t="s">
         <v>29</v>
       </c>
-      <c r="G20" s="1">
+      <c r="H20" s="1">
         <v>0.6430555555555556</v>
       </c>
-      <c r="H20" s="1">
+      <c r="I20" s="1">
         <v>0.64513888888888893</v>
       </c>
-      <c r="I20">
-        <v>0</v>
-      </c>
       <c r="J20">
+        <v>0</v>
+      </c>
+      <c r="K20">
         <v>11</v>
       </c>
-      <c r="K20" t="s">
+      <c r="L20" t="s">
         <v>15</v>
       </c>
-      <c r="L20" t="s">
+      <c r="M20" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1318,26 +1384,29 @@
       <c r="E21" t="s">
         <v>26</v>
       </c>
-      <c r="F21" t="s">
-        <v>22</v>
-      </c>
-      <c r="G21" s="1">
+      <c r="F21">
+        <v>0</v>
+      </c>
+      <c r="G21" t="s">
+        <v>22</v>
+      </c>
+      <c r="H21" s="1">
         <v>0.65416666666666667</v>
       </c>
-      <c r="H21" s="1">
+      <c r="I21" s="1">
         <v>0.65625</v>
       </c>
-      <c r="I21" t="s">
+      <c r="J21" t="s">
         <v>15</v>
-      </c>
-      <c r="J21">
-        <v>7</v>
       </c>
       <c r="K21">
         <v>7</v>
       </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L21">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1353,26 +1422,29 @@
       <c r="E22" t="s">
         <v>26</v>
       </c>
-      <c r="F22" t="s">
-        <v>22</v>
-      </c>
-      <c r="G22" s="1">
+      <c r="F22">
+        <v>0</v>
+      </c>
+      <c r="G22" t="s">
+        <v>22</v>
+      </c>
+      <c r="H22" s="1">
         <v>0.65555555555555556</v>
       </c>
-      <c r="H22" s="1">
+      <c r="I22" s="1">
         <v>0.65625</v>
       </c>
-      <c r="I22" t="s">
+      <c r="J22" t="s">
         <v>15</v>
       </c>
-      <c r="J22">
+      <c r="K22">
         <v>11</v>
       </c>
-      <c r="K22">
+      <c r="L22">
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1388,29 +1460,32 @@
       <c r="E23" t="s">
         <v>26</v>
       </c>
-      <c r="F23" t="s">
-        <v>22</v>
-      </c>
-      <c r="G23" s="1">
-        <v>0.65902777777777777</v>
+      <c r="F23">
+        <v>0</v>
+      </c>
+      <c r="G23" t="s">
+        <v>22</v>
       </c>
       <c r="H23" s="1">
         <v>0.65902777777777777</v>
       </c>
-      <c r="I23">
+      <c r="I23" s="1">
+        <v>0.65902777777777777</v>
+      </c>
+      <c r="J23">
         <v>4</v>
       </c>
-      <c r="J23">
+      <c r="K23">
         <v>10</v>
       </c>
-      <c r="K23">
+      <c r="L23">
         <v>8</v>
       </c>
-      <c r="L23" t="s">
+      <c r="M23" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1426,29 +1501,32 @@
       <c r="E24" t="s">
         <v>26</v>
       </c>
-      <c r="F24" t="s">
-        <v>22</v>
-      </c>
-      <c r="G24" s="1">
+      <c r="F24">
+        <v>0</v>
+      </c>
+      <c r="G24" t="s">
+        <v>22</v>
+      </c>
+      <c r="H24" s="1">
         <v>0.66388888888888886</v>
       </c>
-      <c r="H24" s="1">
+      <c r="I24" s="1">
         <v>0.6645833333333333</v>
       </c>
-      <c r="I24">
+      <c r="J24">
         <v>13</v>
       </c>
-      <c r="J24">
+      <c r="K24">
         <v>20</v>
       </c>
-      <c r="K24">
+      <c r="L24">
         <v>23</v>
       </c>
-      <c r="L24" t="s">
+      <c r="M24" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1464,26 +1542,29 @@
       <c r="E25" t="s">
         <v>26</v>
       </c>
-      <c r="F25" t="s">
-        <v>22</v>
-      </c>
-      <c r="G25" s="1">
+      <c r="F25">
+        <v>0</v>
+      </c>
+      <c r="G25" t="s">
+        <v>22</v>
+      </c>
+      <c r="H25" s="1">
         <v>0.66597222222222219</v>
       </c>
-      <c r="H25" s="1">
+      <c r="I25" s="1">
         <v>0.66527777777777775</v>
       </c>
-      <c r="I25">
+      <c r="J25">
         <v>9</v>
       </c>
-      <c r="J25">
+      <c r="K25">
         <v>4</v>
       </c>
-      <c r="K25">
+      <c r="L25">
         <v>7</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1499,26 +1580,29 @@
       <c r="E26" t="s">
         <v>26</v>
       </c>
-      <c r="F26" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="G26" s="1">
+      <c r="F26">
+        <v>0</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H26" s="1">
         <v>0.66805555555555551</v>
       </c>
-      <c r="H26" s="1">
+      <c r="I26" s="1">
         <v>0.67013888888888884</v>
       </c>
-      <c r="I26" s="5">
+      <c r="J26">
         <v>7</v>
       </c>
-      <c r="J26" s="5">
+      <c r="K26">
         <v>7</v>
       </c>
-      <c r="K26" s="5">
+      <c r="L26">
         <v>13</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1534,26 +1618,29 @@
       <c r="E27" t="s">
         <v>26</v>
       </c>
-      <c r="F27" t="s">
-        <v>22</v>
-      </c>
-      <c r="G27" s="1">
+      <c r="F27">
+        <v>0</v>
+      </c>
+      <c r="G27" t="s">
+        <v>22</v>
+      </c>
+      <c r="H27" s="1">
         <v>0.67291666666666672</v>
       </c>
-      <c r="H27" s="1">
+      <c r="I27" s="1">
         <v>0.67708333333333337</v>
       </c>
-      <c r="I27" s="5">
+      <c r="J27">
         <v>13</v>
       </c>
-      <c r="J27" s="5">
+      <c r="K27">
         <v>4</v>
       </c>
-      <c r="K27" s="5">
+      <c r="L27">
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1569,26 +1656,29 @@
       <c r="E28" t="s">
         <v>26</v>
       </c>
-      <c r="F28" t="s">
-        <v>22</v>
-      </c>
-      <c r="G28" s="1">
+      <c r="F28">
+        <v>0</v>
+      </c>
+      <c r="G28" t="s">
+        <v>22</v>
+      </c>
+      <c r="H28" s="1">
         <v>0.67986111111111114</v>
       </c>
-      <c r="H28" s="1">
+      <c r="I28" s="1">
         <v>0.6791666666666667</v>
       </c>
-      <c r="I28" s="5">
+      <c r="J28">
         <v>3</v>
       </c>
-      <c r="J28" s="5">
+      <c r="K28">
         <v>5</v>
       </c>
-      <c r="K28" t="s">
+      <c r="L28" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1604,29 +1694,32 @@
       <c r="E29" t="s">
         <v>26</v>
       </c>
-      <c r="F29" t="s">
-        <v>22</v>
-      </c>
-      <c r="G29" s="1">
+      <c r="F29">
+        <v>0</v>
+      </c>
+      <c r="G29" t="s">
+        <v>22</v>
+      </c>
+      <c r="H29" s="1">
         <v>0.67847222222222225</v>
       </c>
-      <c r="H29" s="1">
+      <c r="I29" s="1">
         <v>0.68055555555555558</v>
       </c>
-      <c r="I29" s="5">
+      <c r="J29">
         <v>2</v>
       </c>
-      <c r="J29" s="5">
+      <c r="K29">
         <v>20</v>
       </c>
-      <c r="K29" t="s">
+      <c r="L29" t="s">
         <v>15</v>
       </c>
-      <c r="L29" t="s">
+      <c r="M29" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1642,26 +1735,29 @@
       <c r="E30" t="s">
         <v>28</v>
       </c>
-      <c r="F30" t="s">
+      <c r="F30">
+        <v>15356</v>
+      </c>
+      <c r="G30" t="s">
         <v>37</v>
-      </c>
-      <c r="G30" s="1">
-        <v>0.46597222222222223</v>
       </c>
       <c r="H30" s="1">
         <v>0.46597222222222223</v>
       </c>
-      <c r="I30" t="s">
+      <c r="I30" s="1">
+        <v>0.46597222222222223</v>
+      </c>
+      <c r="J30" t="s">
         <v>15</v>
       </c>
-      <c r="J30" s="5">
+      <c r="K30">
         <v>2</v>
       </c>
-      <c r="K30" s="5">
+      <c r="L30">
         <v>3</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1677,29 +1773,32 @@
       <c r="E31" t="s">
         <v>28</v>
       </c>
-      <c r="F31" t="s">
+      <c r="F31">
+        <v>15356</v>
+      </c>
+      <c r="G31" t="s">
         <v>37</v>
       </c>
-      <c r="G31" s="1">
+      <c r="H31" s="1">
         <v>0.46736111111111112</v>
       </c>
-      <c r="H31" s="1">
+      <c r="I31" s="1">
         <v>0.46875</v>
       </c>
-      <c r="I31">
+      <c r="J31">
         <v>3</v>
       </c>
-      <c r="J31" s="5">
+      <c r="K31">
         <v>11</v>
       </c>
-      <c r="K31" s="5">
+      <c r="L31">
         <v>11</v>
       </c>
-      <c r="L31" t="s">
+      <c r="M31" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1715,26 +1814,29 @@
       <c r="E32" t="s">
         <v>28</v>
       </c>
-      <c r="F32" t="s">
+      <c r="F32">
+        <v>15356</v>
+      </c>
+      <c r="G32" t="s">
         <v>37</v>
-      </c>
-      <c r="G32" s="1">
-        <v>0.47638888888888886</v>
       </c>
       <c r="H32" s="1">
         <v>0.47638888888888886</v>
       </c>
-      <c r="I32">
+      <c r="I32" s="1">
+        <v>0.47638888888888886</v>
+      </c>
+      <c r="J32">
         <v>11</v>
       </c>
-      <c r="J32" s="5">
+      <c r="K32">
         <v>9</v>
       </c>
-      <c r="K32" s="5">
+      <c r="L32">
         <v>9</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1750,29 +1852,32 @@
       <c r="E33" t="s">
         <v>28</v>
       </c>
-      <c r="F33" t="s">
+      <c r="F33">
+        <v>15356</v>
+      </c>
+      <c r="G33" t="s">
         <v>37</v>
-      </c>
-      <c r="G33" s="1">
-        <v>0.4826388888888889</v>
       </c>
       <c r="H33" s="1">
         <v>0.4826388888888889</v>
       </c>
-      <c r="I33">
+      <c r="I33" s="1">
+        <v>0.4826388888888889</v>
+      </c>
+      <c r="J33">
         <v>9</v>
       </c>
-      <c r="J33" s="5">
+      <c r="K33">
         <v>10</v>
       </c>
-      <c r="K33" s="5">
+      <c r="L33">
         <v>14</v>
       </c>
-      <c r="L33" t="s">
+      <c r="M33" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1788,25 +1893,28 @@
       <c r="E34" t="s">
         <v>28</v>
       </c>
-      <c r="F34" t="s">
+      <c r="F34">
+        <v>15356</v>
+      </c>
+      <c r="G34" t="s">
         <v>37</v>
       </c>
-      <c r="G34" s="1">
+      <c r="H34" s="1">
         <v>0.48958333333333331</v>
       </c>
-      <c r="H34" s="1">
+      <c r="I34" s="1">
         <v>0.49236111111111114</v>
       </c>
-      <c r="I34">
+      <c r="J34">
         <v>14</v>
       </c>
-      <c r="J34" s="5">
+      <c r="K34">
         <v>5</v>
       </c>
-      <c r="K34" t="s">
+      <c r="L34" t="s">
         <v>15</v>
       </c>
-      <c r="L34" t="s">
+      <c r="M34" t="s">
         <v>34</v>
       </c>
     </row>

</xml_diff>